<commit_message>
Excel de PI: etiquetar las curvas de 25 a 45 m como radio excepcional
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AQK5QV5EuwJ2d1eMj5feZi
</commit_message>
<xml_diff>
--- a/informes/PI_eje_DG2018_tramo_1080-4500.xlsx
+++ b/informes/PI_eje_DG2018_tramo_1080-4500.xlsx
@@ -502,7 +502,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Coordenadas UTM WGS84 zona 17 Sur. Sentido D = derecha, I = izquierda. Sombreado amarillo = curva excepcional (25 ≤ R &lt; 45 m, Ve = 30 km/h); naranja = curva de vuelta (R &lt; 25 m).</t>
+          <t>Coordenadas UTM WGS84 zona 17 Sur. Sentido D = derecha, I = izquierda. Sombreado amarillo = radio excepcional (25 ≤ R &lt; 45 m); naranja = curva de vuelta (R &lt; 25 m).</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K12" s="10" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K14" s="10" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K16" s="10" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="J17" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K17" s="10" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K25" s="10" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K29" s="10" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K33" s="10" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K41" s="10" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="J42" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K42" s="10" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="J48" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K48" s="10" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="J52" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K52" s="10" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="J55" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K55" s="10" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="J63" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K63" s="10" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="J68" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K68" s="10" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="J71" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K71" s="10" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="J72" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K72" s="10" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="J89" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K89" s="10" t="inlineStr">
@@ -4778,7 +4778,7 @@
       </c>
       <c r="J92" s="10" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="K92" s="10" t="inlineStr">
@@ -5102,7 +5102,7 @@
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Excepcional (Ve = 30 km/h)</t>
+          <t>Radio excepcional (25 ≤ R &lt; 45 m)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -5110,7 +5110,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>25 ≤ R &lt; 45 m: velocidad específica 30 km/h (Tópico 204.03 y fila de 30 km/h de la Tabla 302.02)</t>
+          <t>Radio menor al mínimo de 45 m de la Tabla 302.02; se adopta de forma excepcional para seguir el trazo existente en zona poblada</t>
         </is>
       </c>
     </row>
@@ -5129,6 +5129,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>

</xml_diff>